<commit_message>
another update of data troll face emoji
</commit_message>
<xml_diff>
--- a/datasets/xlsx/CounterStrike2.xlsx
+++ b/datasets/xlsx/CounterStrike2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\avery\OneDrive\Desktop\Programming SHit\HardWareWebsite\datasets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CA49B24-BFE7-4E03-AB2D-4381EB541B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E76625E-0C17-4048-9CFC-CF45F5F6CBE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-24120" yWindow="7890" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -159,7 +159,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7180" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7187" uniqueCount="120">
   <si>
     <t>ID</t>
   </si>
@@ -100403,6 +100403,72 @@
       </c>
     </row>
     <row r="1158" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A1158">
+        <v>1157</v>
+      </c>
+      <c r="B1158">
+        <v>2</v>
+      </c>
+      <c r="C1158" s="1">
+        <v>46295</v>
+      </c>
+      <c r="D1158" s="2">
+        <v>0.83402777777777781</v>
+      </c>
+      <c r="E1158" s="2">
+        <v>0.83402777777777781</v>
+      </c>
+      <c r="F1158" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1158" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1158" t="s">
+        <v>60</v>
+      </c>
+      <c r="I1158" t="s">
+        <v>104</v>
+      </c>
+      <c r="J1158" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1158">
+        <v>15</v>
+      </c>
+      <c r="L1158">
+        <v>3</v>
+      </c>
+      <c r="M1158">
+        <v>10</v>
+      </c>
+      <c r="N1158">
+        <v>15</v>
+      </c>
+      <c r="O1158">
+        <v>5</v>
+      </c>
+      <c r="P1158">
+        <v>6</v>
+      </c>
+      <c r="Q1158">
+        <v>2975</v>
+      </c>
+      <c r="R1158">
+        <v>102</v>
+      </c>
+      <c r="S1158">
+        <v>33</v>
+      </c>
+      <c r="T1158" t="s">
+        <v>63</v>
+      </c>
+      <c r="U1158" t="s">
+        <v>108</v>
+      </c>
+      <c r="V1158">
+        <v>2</v>
+      </c>
       <c r="AC1158">
         <f t="shared" si="144"/>
         <v>1</v>
@@ -100413,13 +100479,13 @@
       </c>
       <c r="AE1158">
         <f t="shared" si="146"/>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1159" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1159">
         <f t="shared" si="144"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD1159">
         <f t="shared" si="145"/>
@@ -100433,7 +100499,7 @@
     <row r="1160" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1160">
         <f t="shared" si="144"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AD1160">
         <f t="shared" si="145"/>
@@ -100447,7 +100513,7 @@
     <row r="1161" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1161">
         <f t="shared" si="144"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AD1161">
         <f t="shared" si="145"/>
@@ -100461,7 +100527,7 @@
     <row r="1162" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1162">
         <f t="shared" si="144"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AD1162">
         <f t="shared" si="145"/>
@@ -100475,7 +100541,7 @@
     <row r="1163" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1163">
         <f t="shared" si="144"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AD1163">
         <f t="shared" si="145"/>
@@ -100489,7 +100555,7 @@
     <row r="1164" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1164">
         <f t="shared" si="144"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AD1164">
         <f t="shared" si="145"/>
@@ -100503,7 +100569,7 @@
     <row r="1165" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1165">
         <f t="shared" si="144"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AD1165">
         <f t="shared" si="145"/>
@@ -100517,7 +100583,7 @@
     <row r="1166" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1166">
         <f t="shared" si="144"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AD1166">
         <f t="shared" si="145"/>
@@ -100531,7 +100597,7 @@
     <row r="1167" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1167">
         <f t="shared" si="144"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AD1167">
         <f t="shared" si="145"/>
@@ -100545,7 +100611,7 @@
     <row r="1168" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1168">
         <f t="shared" si="144"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AD1168">
         <f t="shared" si="145"/>
@@ -100559,7 +100625,7 @@
     <row r="1169" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1169">
         <f t="shared" si="144"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AD1169">
         <f t="shared" si="145"/>
@@ -100573,7 +100639,7 @@
     <row r="1170" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1170">
         <f t="shared" si="144"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AD1170">
         <f t="shared" si="145"/>
@@ -100587,7 +100653,7 @@
     <row r="1171" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1171">
         <f t="shared" si="144"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AD1171">
         <f t="shared" si="145"/>
@@ -100601,7 +100667,7 @@
     <row r="1172" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1172">
         <f t="shared" si="144"/>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AD1172">
         <f t="shared" si="145"/>
@@ -100615,7 +100681,7 @@
     <row r="1173" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1173">
         <f t="shared" si="144"/>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AD1173">
         <f t="shared" si="145"/>
@@ -100629,7 +100695,7 @@
     <row r="1174" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1174">
         <f t="shared" si="144"/>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="AD1174">
         <f t="shared" si="145"/>
@@ -100643,7 +100709,7 @@
     <row r="1175" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1175">
         <f t="shared" si="144"/>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AD1175">
         <f t="shared" si="145"/>
@@ -100657,7 +100723,7 @@
     <row r="1176" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1176">
         <f t="shared" si="144"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AD1176">
         <f t="shared" si="145"/>
@@ -100671,7 +100737,7 @@
     <row r="1177" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1177">
         <f t="shared" si="144"/>
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AD1177">
         <f t="shared" si="145"/>
@@ -100685,7 +100751,7 @@
     <row r="1178" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1178">
         <f t="shared" si="144"/>
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="AD1178">
         <f t="shared" si="145"/>
@@ -100699,7 +100765,7 @@
     <row r="1179" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1179">
         <f t="shared" si="144"/>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="AD1179">
         <f t="shared" si="145"/>
@@ -100713,7 +100779,7 @@
     <row r="1180" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1180">
         <f t="shared" si="144"/>
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="AD1180">
         <f t="shared" si="145"/>
@@ -100727,7 +100793,7 @@
     <row r="1181" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1181">
         <f t="shared" si="144"/>
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="AD1181">
         <f t="shared" si="145"/>
@@ -100741,7 +100807,7 @@
     <row r="1182" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1182">
         <f t="shared" si="144"/>
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="AD1182">
         <f t="shared" si="145"/>
@@ -100755,7 +100821,7 @@
     <row r="1183" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1183">
         <f t="shared" si="144"/>
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="AD1183">
         <f t="shared" si="145"/>
@@ -100769,7 +100835,7 @@
     <row r="1184" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1184">
         <f t="shared" si="144"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="AD1184">
         <f t="shared" si="145"/>
@@ -100783,7 +100849,7 @@
     <row r="1185" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1185">
         <f t="shared" si="144"/>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="AD1185">
         <f t="shared" si="145"/>
@@ -100797,7 +100863,7 @@
     <row r="1186" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1186">
         <f t="shared" si="144"/>
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="AD1186">
         <f t="shared" si="145"/>

</xml_diff>

<commit_message>
im hoping updated data
</commit_message>
<xml_diff>
--- a/datasets/xlsx/CounterStrike2.xlsx
+++ b/datasets/xlsx/CounterStrike2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\avery\OneDrive\Desktop\Programming SHit\HardWareWebsite\datasets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E76625E-0C17-4048-9CFC-CF45F5F6CBE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{326EA3A4-92EC-4D8B-A9E6-E633D1E644E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-24120" yWindow="7890" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -159,7 +159,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7187" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7205" uniqueCount="120">
   <si>
     <t>ID</t>
   </si>
@@ -100483,6 +100483,72 @@
       </c>
     </row>
     <row r="1159" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A1159">
+        <v>1158</v>
+      </c>
+      <c r="B1159">
+        <v>1</v>
+      </c>
+      <c r="C1159" s="1">
+        <v>46299</v>
+      </c>
+      <c r="D1159" s="2">
+        <v>0.89652777777777781</v>
+      </c>
+      <c r="E1159" s="2">
+        <v>0.89652777777777781</v>
+      </c>
+      <c r="F1159" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1159" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1159" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1159" t="s">
+        <v>64</v>
+      </c>
+      <c r="J1159" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1159">
+        <v>5</v>
+      </c>
+      <c r="L1159">
+        <v>7</v>
+      </c>
+      <c r="M1159">
+        <v>8</v>
+      </c>
+      <c r="N1159">
+        <v>10</v>
+      </c>
+      <c r="O1159">
+        <v>1</v>
+      </c>
+      <c r="P1159">
+        <v>7</v>
+      </c>
+      <c r="Q1159">
+        <v>1987</v>
+      </c>
+      <c r="R1159">
+        <v>86</v>
+      </c>
+      <c r="S1159">
+        <v>33</v>
+      </c>
+      <c r="T1159" t="s">
+        <v>63</v>
+      </c>
+      <c r="U1159">
+        <v>17651</v>
+      </c>
+      <c r="V1159">
+        <v>1</v>
+      </c>
       <c r="AC1159">
         <f t="shared" si="144"/>
         <v>1</v>
@@ -100493,17 +100559,83 @@
       </c>
       <c r="AE1159">
         <f t="shared" si="146"/>
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="1160" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A1160">
+        <v>1159</v>
+      </c>
+      <c r="B1160">
+        <v>1</v>
+      </c>
+      <c r="C1160" s="1">
+        <v>46305</v>
+      </c>
+      <c r="D1160" s="2">
+        <v>0.81388888888888888</v>
+      </c>
+      <c r="E1160" s="2">
+        <v>0.81388888888888888</v>
+      </c>
+      <c r="F1160" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1160" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1160" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1160" t="s">
+        <v>87</v>
+      </c>
+      <c r="J1160" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1160">
+        <v>5</v>
+      </c>
+      <c r="L1160">
+        <v>3</v>
+      </c>
+      <c r="M1160">
+        <v>8</v>
+      </c>
+      <c r="N1160">
+        <v>5</v>
+      </c>
+      <c r="O1160">
+        <v>2</v>
+      </c>
+      <c r="P1160">
+        <v>7</v>
+      </c>
+      <c r="Q1160">
+        <v>1147</v>
+      </c>
+      <c r="R1160">
+        <v>54</v>
+      </c>
+      <c r="S1160">
+        <v>50</v>
+      </c>
+      <c r="T1160" t="s">
+        <v>58</v>
+      </c>
+      <c r="U1160">
+        <v>18119</v>
+      </c>
+      <c r="V1160">
+        <v>1</v>
+      </c>
       <c r="AC1160">
         <f t="shared" si="144"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD1160">
         <f t="shared" si="145"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE1160">
         <f t="shared" si="146"/>
@@ -100511,9 +100643,75 @@
       </c>
     </row>
     <row r="1161" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A1161">
+        <v>1160</v>
+      </c>
+      <c r="B1161">
+        <v>1</v>
+      </c>
+      <c r="C1161" s="1">
+        <v>46305</v>
+      </c>
+      <c r="D1161" s="2">
+        <v>0.84375</v>
+      </c>
+      <c r="E1161" s="2">
+        <v>0.84375</v>
+      </c>
+      <c r="F1161" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1161" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1161" t="s">
+        <v>60</v>
+      </c>
+      <c r="I1161" t="s">
+        <v>87</v>
+      </c>
+      <c r="J1161" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1161">
+        <v>3</v>
+      </c>
+      <c r="L1161">
+        <v>2</v>
+      </c>
+      <c r="M1161">
+        <v>3</v>
+      </c>
+      <c r="N1161">
+        <v>10</v>
+      </c>
+      <c r="O1161">
+        <v>4</v>
+      </c>
+      <c r="P1161">
+        <v>8</v>
+      </c>
+      <c r="Q1161">
+        <v>1374</v>
+      </c>
+      <c r="R1161">
+        <v>72</v>
+      </c>
+      <c r="S1161">
+        <v>46</v>
+      </c>
+      <c r="T1161" t="s">
+        <v>63</v>
+      </c>
+      <c r="U1161">
+        <v>18005</v>
+      </c>
+      <c r="V1161">
+        <v>1</v>
+      </c>
       <c r="AC1161">
         <f t="shared" si="144"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AD1161">
         <f t="shared" si="145"/>
@@ -100521,13 +100719,13 @@
       </c>
       <c r="AE1161">
         <f t="shared" si="146"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1162" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1162">
         <f t="shared" si="144"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AD1162">
         <f t="shared" si="145"/>
@@ -100541,7 +100739,7 @@
     <row r="1163" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1163">
         <f t="shared" si="144"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AD1163">
         <f t="shared" si="145"/>
@@ -100555,7 +100753,7 @@
     <row r="1164" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1164">
         <f t="shared" si="144"/>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AD1164">
         <f t="shared" si="145"/>
@@ -100569,7 +100767,7 @@
     <row r="1165" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1165">
         <f t="shared" si="144"/>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AD1165">
         <f t="shared" si="145"/>
@@ -100583,7 +100781,7 @@
     <row r="1166" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1166">
         <f t="shared" si="144"/>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="AD1166">
         <f t="shared" si="145"/>
@@ -100597,7 +100795,7 @@
     <row r="1167" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1167">
         <f t="shared" si="144"/>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="AD1167">
         <f t="shared" si="145"/>
@@ -100611,7 +100809,7 @@
     <row r="1168" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1168">
         <f t="shared" si="144"/>
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="AD1168">
         <f t="shared" si="145"/>
@@ -100625,7 +100823,7 @@
     <row r="1169" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1169">
         <f t="shared" si="144"/>
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="AD1169">
         <f t="shared" si="145"/>
@@ -100639,7 +100837,7 @@
     <row r="1170" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1170">
         <f t="shared" si="144"/>
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="AD1170">
         <f t="shared" si="145"/>
@@ -100653,7 +100851,7 @@
     <row r="1171" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1171">
         <f t="shared" si="144"/>
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="AD1171">
         <f t="shared" si="145"/>
@@ -100667,7 +100865,7 @@
     <row r="1172" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1172">
         <f t="shared" si="144"/>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="AD1172">
         <f t="shared" si="145"/>
@@ -100681,7 +100879,7 @@
     <row r="1173" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1173">
         <f t="shared" si="144"/>
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="AD1173">
         <f t="shared" si="145"/>
@@ -100695,7 +100893,7 @@
     <row r="1174" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1174">
         <f t="shared" si="144"/>
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="AD1174">
         <f t="shared" si="145"/>
@@ -100709,7 +100907,7 @@
     <row r="1175" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1175">
         <f t="shared" si="144"/>
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="AD1175">
         <f t="shared" si="145"/>
@@ -100723,7 +100921,7 @@
     <row r="1176" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1176">
         <f t="shared" si="144"/>
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="AD1176">
         <f t="shared" si="145"/>
@@ -100737,7 +100935,7 @@
     <row r="1177" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1177">
         <f t="shared" si="144"/>
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="AD1177">
         <f t="shared" si="145"/>
@@ -100751,7 +100949,7 @@
     <row r="1178" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1178">
         <f t="shared" si="144"/>
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="AD1178">
         <f t="shared" si="145"/>
@@ -100765,7 +100963,7 @@
     <row r="1179" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1179">
         <f t="shared" si="144"/>
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="AD1179">
         <f t="shared" si="145"/>
@@ -100779,7 +100977,7 @@
     <row r="1180" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1180">
         <f t="shared" si="144"/>
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="AD1180">
         <f t="shared" si="145"/>
@@ -100793,7 +100991,7 @@
     <row r="1181" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1181">
         <f t="shared" si="144"/>
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="AD1181">
         <f t="shared" si="145"/>
@@ -100807,7 +101005,7 @@
     <row r="1182" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1182">
         <f t="shared" si="144"/>
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="AD1182">
         <f t="shared" si="145"/>
@@ -100821,7 +101019,7 @@
     <row r="1183" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1183">
         <f t="shared" si="144"/>
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="AD1183">
         <f t="shared" si="145"/>
@@ -100835,7 +101033,7 @@
     <row r="1184" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1184">
         <f t="shared" si="144"/>
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="AD1184">
         <f t="shared" si="145"/>
@@ -100849,7 +101047,7 @@
     <row r="1185" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1185">
         <f t="shared" si="144"/>
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="AD1185">
         <f t="shared" si="145"/>
@@ -100863,7 +101061,7 @@
     <row r="1186" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1186">
         <f t="shared" si="144"/>
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="AD1186">
         <f t="shared" si="145"/>

</xml_diff>

<commit_message>
update data again lol
</commit_message>
<xml_diff>
--- a/datasets/xlsx/CounterStrike2.xlsx
+++ b/datasets/xlsx/CounterStrike2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\avery\OneDrive\Desktop\Programming SHit\HardWareWebsite\datasets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{326EA3A4-92EC-4D8B-A9E6-E633D1E644E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{339E75B7-2964-43B5-9E46-09AC8D9535A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-24120" yWindow="7890" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,6 +54,7 @@
     <author>tc={D9F86935-42F8-4EAB-96F7-0BFAB0E14651}</author>
     <author>tc={0A885350-D4D6-4082-BA12-BE8887503B81}</author>
     <author>tc={659DF264-58B9-45A3-8F8E-9E29862B41EA}</author>
+    <author>tc={191C6643-5D71-41D2-B241-FBFD190B6F26}</author>
   </authors>
   <commentList>
     <comment ref="Q8" authorId="0" shapeId="0" xr:uid="{7445B883-AF40-450E-997B-6591AE177020}">
@@ -154,12 +155,20 @@
     Forgot to roll a random number and follow it ☹️</t>
       </text>
     </comment>
+    <comment ref="AA1162" authorId="12" shapeId="0" xr:uid="{191C6643-5D71-41D2-B241-FBFD190B6F26}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Rare vacnet ban</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7205" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7217" uniqueCount="120">
   <si>
     <t>ID</t>
   </si>
@@ -525,13 +534,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -601,6 +616,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Alex Post" id="{5EB933F9-0E4F-489B-95EE-F89F826848D9}" userId="09da2d7264e3c107" providerId="Windows Live"/>
   <person displayName="Post, Alex Michael" id="{9D2E1210-4F23-435E-9530-FBAC86359921}" userId="S::apost7@rockets.utoledo.edu::a051696b-502b-4221-9702-a6ddd3fc6347" providerId="AD"/>
 </personList>
 </file>
@@ -956,6 +972,9 @@
   <threadedComment ref="G807" dT="2025-09-03T02:13:19.22" personId="{9D2E1210-4F23-435E-9530-FBAC86359921}" id="{659DF264-58B9-45A3-8F8E-9E29862B41EA}">
     <text>Forgot to roll a random number and follow it ☹️</text>
   </threadedComment>
+  <threadedComment ref="AA1162" dT="2026-10-13T02:03:35.39" personId="{5EB933F9-0E4F-489B-95EE-F89F826848D9}" id="{191C6643-5D71-41D2-B241-FBFD190B6F26}">
+    <text>Rare vacnet ban</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
@@ -100723,6 +100742,63 @@
       </c>
     </row>
     <row r="1162" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A1162">
+        <v>1161</v>
+      </c>
+      <c r="B1162">
+        <v>1</v>
+      </c>
+      <c r="C1162" s="1">
+        <v>46307</v>
+      </c>
+      <c r="D1162" s="2">
+        <v>0.90972222222222221</v>
+      </c>
+      <c r="E1162" s="2">
+        <v>0.90972222222222221</v>
+      </c>
+      <c r="F1162" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1162" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1162" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1162" t="s">
+        <v>87</v>
+      </c>
+      <c r="J1162" t="s">
+        <v>57</v>
+      </c>
+      <c r="K1162">
+        <v>7</v>
+      </c>
+      <c r="L1162">
+        <v>3</v>
+      </c>
+      <c r="M1162">
+        <v>2</v>
+      </c>
+      <c r="N1162">
+        <v>0</v>
+      </c>
+      <c r="O1162">
+        <v>0</v>
+      </c>
+      <c r="P1162">
+        <v>0</v>
+      </c>
+      <c r="U1162">
+        <v>18456</v>
+      </c>
+      <c r="V1162">
+        <v>1</v>
+      </c>
+      <c r="AA1162" t="s">
+        <v>71</v>
+      </c>
       <c r="AC1162">
         <f t="shared" si="144"/>
         <v>1</v>
@@ -100737,13 +100813,79 @@
       </c>
     </row>
     <row r="1163" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A1163">
+        <v>1162</v>
+      </c>
+      <c r="B1163">
+        <v>1</v>
+      </c>
+      <c r="C1163" s="1">
+        <v>46307</v>
+      </c>
+      <c r="D1163" s="2">
+        <v>0.92083333333333328</v>
+      </c>
+      <c r="E1163" s="2">
+        <v>0.92083333333333328</v>
+      </c>
+      <c r="F1163" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1163" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1163" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1163" t="s">
+        <v>104</v>
+      </c>
+      <c r="J1163" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1163">
+        <v>5</v>
+      </c>
+      <c r="L1163">
+        <v>1</v>
+      </c>
+      <c r="M1163">
+        <v>11</v>
+      </c>
+      <c r="N1163">
+        <v>9</v>
+      </c>
+      <c r="O1163">
+        <v>3</v>
+      </c>
+      <c r="P1163">
+        <v>7</v>
+      </c>
+      <c r="Q1163">
+        <v>1616</v>
+      </c>
+      <c r="R1163">
+        <v>67</v>
+      </c>
+      <c r="S1163">
+        <v>35</v>
+      </c>
+      <c r="T1163" t="s">
+        <v>58</v>
+      </c>
+      <c r="U1163">
+        <v>18456</v>
+      </c>
+      <c r="V1163">
+        <v>2</v>
+      </c>
       <c r="AC1163">
         <f t="shared" si="144"/>
         <v>2</v>
       </c>
       <c r="AD1163">
         <f t="shared" si="145"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE1163">
         <f t="shared" si="146"/>
@@ -100753,7 +100895,7 @@
     <row r="1164" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1164">
         <f t="shared" si="144"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AD1164">
         <f t="shared" si="145"/>
@@ -100767,7 +100909,7 @@
     <row r="1165" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1165">
         <f t="shared" si="144"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AD1165">
         <f t="shared" si="145"/>
@@ -100781,7 +100923,7 @@
     <row r="1166" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1166">
         <f t="shared" si="144"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AD1166">
         <f t="shared" si="145"/>
@@ -100795,7 +100937,7 @@
     <row r="1167" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1167">
         <f t="shared" si="144"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AD1167">
         <f t="shared" si="145"/>
@@ -100809,7 +100951,7 @@
     <row r="1168" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1168">
         <f t="shared" si="144"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD1168">
         <f t="shared" si="145"/>
@@ -100823,7 +100965,7 @@
     <row r="1169" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1169">
         <f t="shared" si="144"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AD1169">
         <f t="shared" si="145"/>
@@ -100837,7 +100979,7 @@
     <row r="1170" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1170">
         <f t="shared" si="144"/>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AD1170">
         <f t="shared" si="145"/>
@@ -100851,7 +100993,7 @@
     <row r="1171" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1171">
         <f t="shared" si="144"/>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AD1171">
         <f t="shared" si="145"/>
@@ -100865,7 +101007,7 @@
     <row r="1172" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1172">
         <f t="shared" si="144"/>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="AD1172">
         <f t="shared" si="145"/>
@@ -100879,7 +101021,7 @@
     <row r="1173" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1173">
         <f t="shared" si="144"/>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AD1173">
         <f t="shared" si="145"/>
@@ -100893,7 +101035,7 @@
     <row r="1174" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1174">
         <f t="shared" si="144"/>
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="AD1174">
         <f t="shared" si="145"/>
@@ -100907,7 +101049,7 @@
     <row r="1175" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1175">
         <f t="shared" si="144"/>
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="AD1175">
         <f t="shared" si="145"/>
@@ -100921,7 +101063,7 @@
     <row r="1176" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1176">
         <f t="shared" si="144"/>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="AD1176">
         <f t="shared" si="145"/>
@@ -100935,7 +101077,7 @@
     <row r="1177" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1177">
         <f t="shared" si="144"/>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="AD1177">
         <f t="shared" si="145"/>
@@ -100949,7 +101091,7 @@
     <row r="1178" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1178">
         <f t="shared" si="144"/>
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="AD1178">
         <f t="shared" si="145"/>
@@ -100963,7 +101105,7 @@
     <row r="1179" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1179">
         <f t="shared" si="144"/>
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="AD1179">
         <f t="shared" si="145"/>
@@ -100977,7 +101119,7 @@
     <row r="1180" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1180">
         <f t="shared" si="144"/>
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="AD1180">
         <f t="shared" si="145"/>
@@ -100991,7 +101133,7 @@
     <row r="1181" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1181">
         <f t="shared" si="144"/>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="AD1181">
         <f t="shared" si="145"/>
@@ -101005,7 +101147,7 @@
     <row r="1182" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1182">
         <f t="shared" si="144"/>
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="AD1182">
         <f t="shared" si="145"/>
@@ -101019,7 +101161,7 @@
     <row r="1183" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1183">
         <f t="shared" si="144"/>
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="AD1183">
         <f t="shared" si="145"/>
@@ -101033,7 +101175,7 @@
     <row r="1184" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1184">
         <f t="shared" si="144"/>
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AD1184">
         <f t="shared" si="145"/>
@@ -101047,7 +101189,7 @@
     <row r="1185" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1185">
         <f t="shared" si="144"/>
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="AD1185">
         <f t="shared" si="145"/>
@@ -101061,7 +101203,7 @@
     <row r="1186" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1186">
         <f t="shared" si="144"/>
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="AD1186">
         <f t="shared" si="145"/>

</xml_diff>

<commit_message>
blue-ska-doo, we can too! update the data.
</commit_message>
<xml_diff>
--- a/datasets/xlsx/CounterStrike2.xlsx
+++ b/datasets/xlsx/CounterStrike2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\avery\OneDrive\Desktop\Programming SHit\HardWareWebsite\datasets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF46CD4D-3B2A-4FA8-937A-375B3D7ABC3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28632B61-7B4E-4F84-B66D-A0998CB181D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-24120" yWindow="7890" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -168,7 +168,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7248" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7260" uniqueCount="120">
   <si>
     <t>ID</t>
   </si>
@@ -101280,10 +101280,76 @@
         <v>1</v>
       </c>
     </row>
-    <row r="1169" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1169" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A1169">
+        <v>1168</v>
+      </c>
+      <c r="B1169">
+        <v>1</v>
+      </c>
+      <c r="C1169" s="1">
+        <v>46310</v>
+      </c>
+      <c r="D1169" s="2">
+        <v>0.83194444444444449</v>
+      </c>
+      <c r="E1169" s="2">
+        <v>0.83194444444444449</v>
+      </c>
+      <c r="F1169" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1169" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1169" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1169" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1169" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1169">
+        <v>5</v>
+      </c>
+      <c r="L1169">
+        <v>4</v>
+      </c>
+      <c r="M1169">
+        <v>3</v>
+      </c>
+      <c r="N1169">
+        <v>5</v>
+      </c>
+      <c r="O1169">
+        <v>5</v>
+      </c>
+      <c r="P1169">
+        <v>5</v>
+      </c>
+      <c r="Q1169">
+        <v>1282</v>
+      </c>
+      <c r="R1169">
+        <v>71</v>
+      </c>
+      <c r="S1169">
+        <v>30</v>
+      </c>
+      <c r="T1169" t="s">
+        <v>63</v>
+      </c>
+      <c r="U1169">
+        <v>19999</v>
+      </c>
+      <c r="V1169">
+        <v>1</v>
+      </c>
       <c r="AC1169">
         <f t="shared" si="144"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AD1169">
         <f t="shared" si="145"/>
@@ -101291,27 +101357,93 @@
       </c>
       <c r="AE1169">
         <f t="shared" si="146"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="1170" spans="29:31" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1170" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A1170">
+        <v>1169</v>
+      </c>
+      <c r="B1170">
+        <v>1</v>
+      </c>
+      <c r="C1170" s="1">
+        <v>46313</v>
+      </c>
+      <c r="D1170" s="2">
+        <v>0.89097222222222228</v>
+      </c>
+      <c r="E1170" s="2">
+        <v>0.89097222222222228</v>
+      </c>
+      <c r="F1170" t="s">
+        <v>50</v>
+      </c>
+      <c r="G1170" t="s">
+        <v>97</v>
+      </c>
+      <c r="H1170" t="s">
+        <v>60</v>
+      </c>
+      <c r="I1170" t="s">
+        <v>61</v>
+      </c>
+      <c r="J1170" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1170">
+        <v>4</v>
+      </c>
+      <c r="L1170">
+        <v>1</v>
+      </c>
+      <c r="M1170">
+        <v>6</v>
+      </c>
+      <c r="N1170">
+        <v>4</v>
+      </c>
+      <c r="O1170">
+        <v>1</v>
+      </c>
+      <c r="P1170">
+        <v>11</v>
+      </c>
+      <c r="Q1170">
+        <v>1246</v>
+      </c>
+      <c r="R1170">
+        <v>69</v>
+      </c>
+      <c r="S1170">
+        <v>25</v>
+      </c>
+      <c r="T1170" t="s">
+        <v>58</v>
+      </c>
+      <c r="U1170">
+        <v>20110</v>
+      </c>
+      <c r="V1170">
+        <v>1</v>
+      </c>
       <c r="AC1170">
         <f t="shared" si="144"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AD1170">
         <f t="shared" si="145"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE1170">
         <f t="shared" si="146"/>
         <v>0</v>
       </c>
     </row>
-    <row r="1171" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1171" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC1171">
         <f t="shared" si="144"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AD1171">
         <f t="shared" si="145"/>
@@ -101322,10 +101454,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1172" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1172" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC1172">
         <f t="shared" si="144"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AD1172">
         <f t="shared" si="145"/>
@@ -101336,10 +101468,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1173" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1173" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC1173">
         <f t="shared" si="144"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AD1173">
         <f t="shared" si="145"/>
@@ -101350,10 +101482,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1174" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1174" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC1174">
         <f t="shared" si="144"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AD1174">
         <f t="shared" si="145"/>
@@ -101364,10 +101496,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1175" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1175" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC1175">
         <f t="shared" si="144"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD1175">
         <f t="shared" si="145"/>
@@ -101378,10 +101510,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1176" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1176" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC1176">
         <f t="shared" si="144"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AD1176">
         <f t="shared" si="145"/>
@@ -101392,10 +101524,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1177" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1177" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC1177">
         <f t="shared" si="144"/>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AD1177">
         <f t="shared" si="145"/>
@@ -101406,10 +101538,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1178" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1178" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC1178">
         <f t="shared" si="144"/>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AD1178">
         <f t="shared" si="145"/>
@@ -101420,10 +101552,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1179" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1179" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC1179">
         <f t="shared" si="144"/>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="AD1179">
         <f t="shared" si="145"/>
@@ -101434,10 +101566,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1180" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1180" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC1180">
         <f t="shared" si="144"/>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AD1180">
         <f t="shared" si="145"/>
@@ -101448,10 +101580,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1181" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1181" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC1181">
         <f t="shared" si="144"/>
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="AD1181">
         <f t="shared" si="145"/>
@@ -101462,10 +101594,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1182" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1182" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC1182">
         <f t="shared" si="144"/>
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="AD1182">
         <f t="shared" si="145"/>
@@ -101476,10 +101608,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1183" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1183" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC1183">
         <f t="shared" si="144"/>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="AD1183">
         <f t="shared" si="145"/>
@@ -101490,10 +101622,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1184" spans="29:31" x14ac:dyDescent="0.25">
+    <row r="1184" spans="1:31" x14ac:dyDescent="0.25">
       <c r="AC1184">
         <f t="shared" si="144"/>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="AD1184">
         <f t="shared" si="145"/>
@@ -101507,7 +101639,7 @@
     <row r="1185" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1185">
         <f t="shared" si="144"/>
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="AD1185">
         <f t="shared" si="145"/>
@@ -101521,7 +101653,7 @@
     <row r="1186" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1186">
         <f t="shared" si="144"/>
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="AD1186">
         <f t="shared" si="145"/>

</xml_diff>

<commit_message>
updating the premier matches
</commit_message>
<xml_diff>
--- a/datasets/xlsx/CounterStrike2.xlsx
+++ b/datasets/xlsx/CounterStrike2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\avery\OneDrive\Desktop\Programming SHit\HardWareWebsite\datasets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C2F1FF8-9A52-4990-A97D-76832F1CF3E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CE560E3-C713-4A43-ACB9-FF41E942A48F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="7890" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="7815" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -168,7 +168,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7278" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7290" uniqueCount="120">
   <si>
     <t>ID</t>
   </si>
@@ -101280,7 +101280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="1169" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1169" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1169">
         <v>1168</v>
       </c>
@@ -101360,7 +101360,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="1170" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1170" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1170">
         <v>1169</v>
       </c>
@@ -101440,7 +101440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1171" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1171" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1171">
         <v>1170</v>
       </c>
@@ -101517,7 +101517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1172" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1172" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1172">
         <v>1171</v>
       </c>
@@ -101597,7 +101597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1173" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1173" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1173">
         <v>1172</v>
       </c>
@@ -101677,21 +101677,165 @@
         <v>1</v>
       </c>
     </row>
-    <row r="1174" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1174" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A1174">
+        <v>1173</v>
+      </c>
+      <c r="B1174">
+        <v>1</v>
+      </c>
+      <c r="C1174" s="1">
+        <v>46324</v>
+      </c>
+      <c r="D1174" s="2">
+        <v>0.78819444444444442</v>
+      </c>
+      <c r="E1174" s="2">
+        <v>0.78819444444444442</v>
+      </c>
+      <c r="F1174" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1174" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1174" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1174" t="s">
+        <v>104</v>
+      </c>
+      <c r="J1174" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1174">
+        <v>13</v>
+      </c>
+      <c r="L1174">
+        <v>4</v>
+      </c>
+      <c r="M1174">
+        <v>12</v>
+      </c>
+      <c r="N1174">
+        <v>13</v>
+      </c>
+      <c r="O1174">
+        <v>2</v>
+      </c>
+      <c r="P1174">
+        <v>10</v>
+      </c>
+      <c r="Q1174">
+        <v>2555</v>
+      </c>
+      <c r="R1174">
+        <v>85</v>
+      </c>
+      <c r="S1174">
+        <v>26</v>
+      </c>
+      <c r="T1174" t="s">
+        <v>58</v>
+      </c>
+      <c r="U1174">
+        <v>19999</v>
+      </c>
+      <c r="V1174">
+        <v>2</v>
+      </c>
       <c r="AC1174">
         <f t="shared" si="144"/>
         <v>1</v>
       </c>
       <c r="AD1174">
         <f t="shared" si="145"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE1174">
         <f t="shared" si="146"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="1175" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="AF1174">
+        <v>-0.33</v>
+      </c>
+      <c r="AG1174">
+        <v>22</v>
+      </c>
+      <c r="AH1174">
+        <v>76</v>
+      </c>
+      <c r="AI1174">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="1175" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A1175">
+        <v>1174</v>
+      </c>
+      <c r="B1175">
+        <v>1</v>
+      </c>
+      <c r="C1175" s="1">
+        <v>46324</v>
+      </c>
+      <c r="D1175" s="2">
+        <v>0.83611111111111114</v>
+      </c>
+      <c r="E1175" s="2">
+        <v>0.83611111111111114</v>
+      </c>
+      <c r="F1175" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1175" t="s">
+        <v>101</v>
+      </c>
+      <c r="H1175" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1175" t="s">
+        <v>52</v>
+      </c>
+      <c r="J1175" t="s">
+        <v>57</v>
+      </c>
+      <c r="K1175">
+        <v>6</v>
+      </c>
+      <c r="L1175">
+        <v>0</v>
+      </c>
+      <c r="M1175">
+        <v>11</v>
+      </c>
+      <c r="N1175">
+        <v>10</v>
+      </c>
+      <c r="O1175">
+        <v>3</v>
+      </c>
+      <c r="P1175">
+        <v>2</v>
+      </c>
+      <c r="Q1175">
+        <v>1695</v>
+      </c>
+      <c r="R1175">
+        <v>89</v>
+      </c>
+      <c r="S1175">
+        <v>25</v>
+      </c>
+      <c r="T1175" t="s">
+        <v>63</v>
+      </c>
+      <c r="U1175">
+        <v>19840</v>
+      </c>
+      <c r="V1175">
+        <v>1</v>
+      </c>
       <c r="AC1175">
         <f t="shared" si="144"/>
         <v>2</v>
@@ -101702,13 +101846,13 @@
       </c>
       <c r="AE1175">
         <f t="shared" si="146"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="1176" spans="1:31" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="1176" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1176">
         <f t="shared" si="144"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AD1176">
         <f t="shared" si="145"/>
@@ -101719,10 +101863,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1177" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1177" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1177">
         <f t="shared" si="144"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AD1177">
         <f t="shared" si="145"/>
@@ -101733,10 +101877,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1178" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1178" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1178">
         <f t="shared" si="144"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AD1178">
         <f t="shared" si="145"/>
@@ -101747,10 +101891,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1179" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1179" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1179">
         <f t="shared" si="144"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AD1179">
         <f t="shared" si="145"/>
@@ -101761,10 +101905,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1180" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1180" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1180">
         <f t="shared" si="144"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AD1180">
         <f t="shared" si="145"/>
@@ -101775,10 +101919,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1181" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1181" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1181">
         <f t="shared" si="144"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AD1181">
         <f t="shared" si="145"/>
@@ -101789,10 +101933,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1182" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1182" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1182">
         <f t="shared" si="144"/>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AD1182">
         <f t="shared" si="145"/>
@@ -101803,10 +101947,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1183" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1183" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1183">
         <f t="shared" si="144"/>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AD1183">
         <f t="shared" si="145"/>
@@ -101817,10 +101961,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1184" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1184" spans="1:35" x14ac:dyDescent="0.25">
       <c r="AC1184">
         <f t="shared" si="144"/>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="AD1184">
         <f t="shared" si="145"/>
@@ -101834,7 +101978,7 @@
     <row r="1185" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1185">
         <f t="shared" si="144"/>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AD1185">
         <f t="shared" si="145"/>
@@ -101848,7 +101992,7 @@
     <row r="1186" spans="29:31" x14ac:dyDescent="0.25">
       <c r="AC1186">
         <f t="shared" si="144"/>
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="AD1186">
         <f t="shared" si="145"/>

</xml_diff>